<commit_message>
Pulligny: the two sides were swapped, as confirmed
The incoming record's own coordinates (48.54194, 6.14139) match Wikidata's
Pulligny (Q1099419) to 0.0 km, and that commune is in Meurthe-et-Moselle —
206 km from Jura. The recorded suggestion had the incoming record labelled
Jura and the existing one Meurthe-et-Moselle. Sinai confirmed the swap, so
the two values are exchanged in decisions.json and the warning is retired.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nli-report.xlsx
+++ b/nli-report.xlsx
@@ -10212,23 +10212,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>פוליני (מחוז יורה, צרפת)</t>
+          <t>פוליני (מחוז מרת ומוזל, צרפת)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>פוליני (מחוז מרת ומוזל, צרפת)</t>
+          <t>פוליני (מחוז יורה, צרפת)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>לבדיקה: הרשומה הנכנסת היא Pulligny, ולפי ויקינתונים (Q1099419) היא במחוז מרת ומוזל — ואילו ההצעה מייחסת אותה ליורה. ייתכן ששני הצדדים הוחלפו. יש לאשר לפני שליחה.</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Spell out the Arabic defect, state both findings, retire the one-row tab
לוחביצה carries two unrelated findings and was filed under one of them. The
Arabic heading is "لوخفيت︠س︡ي︠ي︠ي︠ي︠ي︠ي (أوكرانيا)" — ي repeated eight times, because
the Roman form Lokhvyt︠s︡i︠a︡ ties t͡s and i͡a with U+FE20/U+FE21 ligature halves
and the Arabic transliteration treated each half as letter-producing. New
"ממצא נוסף" columns state it in full, with the proposed form and the scope
(1 of 1,188 Arabic headings checked, so a one-off, not a pipeline failure).

North Huntingdon's missing closing bracket moves to the heading-correction
tab, which leaves בודדות empty — 8 tabs now. That tab is no longer
Hebrew-only (North Huntingdon's heading is Roman), so it is retitled
"שגיאה בכותרת עצמה" and its columns "הצורה ברשומה / הצורה המוצעת", and the
bracket fix is stated as a correction rather than left in a note.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nli-report.xlsx
+++ b/nli-report.xlsx
@@ -13,22 +13,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="034 פגום" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מזהה ויקינתונים" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כותרת לשני מקומות" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="איות הכותרת" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תיקון הכותרת" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="זהות הכותרת" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כפילות ברשומות" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בודדות" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הסברים" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הסברים" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'אפס שנשמט'!$A$1:$J$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'קואורדינטות שגויות'!$A$1:$M$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'034 פגום'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'מזהה ויקינתונים'!$A$1:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'מזהה ויקינתונים'!$A$1:$M$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'כותרת לשני מקומות'!$A$1:$M$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'איות הכותרת'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'תיקון הכותרת'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'זהות הכותרת'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'כפילות ברשומות'!$A$1:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'בודדות'!$A$1:$G$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -573,7 +571,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    איות הכותרת — 3 שורות — שגיאה באיות הכותרת העברית</t>
+          <t xml:space="preserve">    תיקון הכותרת — 4 שורות — שגיאה בכותרת עצמה</t>
         </is>
       </c>
     </row>
@@ -592,24 +590,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    בודדות — 1 שורות — תקלות בודדות</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>כל שורה עברה סקירה ידנית. עמודת "הערת הסוקר" נושאת את הממצא</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
-        <is>
-          <t>כל שורה עברה סקירה ידנית. עמודת "הערת הסוקר" נושאת את הממצא</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
         <is>
           <t>כפי שנרשם בעת הסקירה.</t>
         </is>
@@ -626,93 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>כותרת עברית</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>כותרת לטינית</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>מזהה NLI</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>הערת הסוקר</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>נקודת NLI</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>נקודת כימה</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>קישור לרשומה</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>North Huntingdon (Pa. : Township)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>987007562247105171</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>הסוגר הסופי חסר בכותרת.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007562247105171</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -954,22 +859,22 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>איות הכותרת</t>
+          <t>תיקון הכותרת</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>שגיאה באיות הכותרת העברית</t>
+          <t>שגיאה בכותרת עצמה</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>כאן אין עמימות ואין שני מקומות — פשוט האיות העברי של הכותרת שגוי, או שהכותרת מעלה שאלה של זהות. אלה ממצאים שעלו אגב בדיקות אחרות ונרשמו במהלך הסקירה.</t>
+          <t>כאן אין עמימות ואין שני מקומות — הכותרת עצמה פגומה: איות עברי שגוי, סוגר שלא נסגר, או שאלה של זהות. אלה ממצאים שעלו אגב בדיקות אחרות ונרשמו במהלך הסקירה, ולכל אחד מהם תיקון קונקרטי.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>לתקן את האיות לפי העמודה "האיות המוצע", או — במקרה של שטרסבורג — להכריע בשאלה שבעמודת ההסבר.</t>
+          <t>לתקן את הכותרת לפי העמודה "הצורה המוצעת", או — במקרה של שטרסבורג — להכריע בשאלה שבעמודת ההסבר.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1054,43 +959,6 @@
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>כל שורה נושאת את שני המזהים ואת שתי הכותרות.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>בודדות</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>תקלות בודדות</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>מקרים שאינם מצטרפים לתבנית — תקלה בשם הערבי, סוגר שלא נסגר בכותרת, סוגריים שנכנסו להפניה. כל שורה עומדת בזכות עצמה, וההערה שלצדה אומרת מה נמצא.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>לקרוא את ההערה בכל שורה ולתקן בהתאם.</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>אלה מקרים שעלו במהלך סקירת קטגוריות אחרות. חלקם הוכרעו בהרצה מוקדמת יותר, והנתונים שלהם נשלפו מחדש מ־Alma OAI לצורך הדוח הזה.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>עמודת "הערה" היא הממצא עצמו.</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9305,8 +9173,10 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9357,10 +9227,20 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
+          <t>ממצא נוסף</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>פירוט הממצא הנוסף</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
           <t>הערת הסוקר</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>קישור לרשומה</t>
         </is>
@@ -9412,10 +9292,20 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>שם ערבי משובש</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>הכותרת הערבית ברשומה היא "لوخفيت︠س︡ي︠ي︠ي︠ي︠ي︠ي (أوكرانيا)" — האות ي חוזרת שמונה פעמים. מקור התקלה בתעתיק: הצורה הלטינית Lokhvyt︠s︡i︠a︡ משתמשת בסימני חיבור (U+FE20/U+FE21) כדי לקשור t͡s ו־i͡a, וההמרה לערבית התייחסה לכל חצי סימן כאל אות ולכן שכפלה את ي. הצורה המוצעת: "لوخفيتسيا (أوكرانيا)". זו תקלה בודדת — אחת מתוך 1,188 כותרות ערביות שנבדקו.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>בעיה בשם הערבי</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007562429505171</t>
         </is>
@@ -9466,7 +9356,9 @@
         <v>2797.7</v>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007543674705171</t>
         </is>
@@ -9516,12 +9408,14 @@
       <c r="I4" t="n">
         <v>104.5</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
         <is>
           <t>אלה הם שני מקומות שונים: העיר וההר. אם הכוונה לעיר, הויקידאטה הוא Q651583 והשם: הויקידאטה והקואורדינטות הנוכחיות ב-nli הן לא של etters-berg אלא של ettersburg הישוב. אם הכוונה היא להר, ממליצה לשנות את השם לאטרס-ברג (גרמניה: הר) והויקידאטה הוא  Q31547753</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007561549805171</t>
         </is>
@@ -9572,7 +9466,9 @@
         <v>54.8</v>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007546333605171</t>
         </is>
@@ -9619,7 +9515,9 @@
         <v>149.4</v>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007284646705171</t>
         </is>
@@ -9670,7 +9568,9 @@
         <v>852.1</v>
       </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564769205171</t>
         </is>
@@ -9721,7 +9621,9 @@
         <v>726.9</v>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987011433524905171</t>
         </is>
@@ -9768,14 +9670,16 @@
         <v>141.3</v>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007545173905171</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K9"/>
+  <autoFilter ref="A1:M9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10283,7 +10187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10313,12 +10217,12 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>האיות ברשומה</t>
+          <t>הצורה ברשומה</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>האיות המוצע</t>
+          <t>הצורה המוצעת</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -10439,8 +10343,41 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>North Huntingdon (Pa. : Township)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>987007562247105171</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>North Huntingdon (Pa. : Township</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>North Huntingdon (Pa. : Township)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>הסוגר הסופי חסר בכותרת.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987007562247105171</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fold the second finding's detail into the reviewer's note
"פירוט" and "הערת הסוקר" were two columns saying one thing. Only one row in
the report fills either: Lokhvytsia, where the detail explains the whole
Arabic transliteration defect and the note said "בעיה בשם הערבי" — a
restatement of the headline already standing in "ממצא נוסף".

The detail now merges into the note at the row level, so the page and the
workbook both get it from one place, and the note that only repeated the
headline is suppressed through the existing NOTE_OVERRIDE rather than by
guessing at overlap. The wikidata-id sheet goes from 14 columns to 13; the
count of rows carrying a note is unchanged at 16.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nli-report.xlsx
+++ b/nli-report.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'אפס שנשמט'!$A$1:$K$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'קואורדינטות שגויות'!$A$1:$M$107</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'034 פגום'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'מזהה ויקינתונים'!$A$1:$N$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'מזהה ויקינתונים'!$A$1:$M$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'תיקון הכותרת'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'זהות הכותרת'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'כפילות ברשומות'!$A$1:$K$7</definedName>
@@ -9705,7 +9705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9718,10 +9718,9 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="70" customWidth="1" min="11" max="11"/>
-    <col width="52" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9777,20 +9776,15 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>פירוט הממצא הנוסף</t>
+          <t>הערת הסוקר</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>הערת הסוקר</t>
+          <t>קישור לרשומה</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>קישור לרשומה</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>נכלל בדוח מיום</t>
         </is>
@@ -9852,15 +9846,10 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>בעיה בשם הערבי</t>
+          <t>https://www.nli.org.il/he/authorities/987007562429505171</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007562429505171</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -9912,13 +9901,12 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987007543674705171</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007543674705171</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -9969,18 +9957,17 @@
         <v>104.5</v>
       </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>אלה הם שני מקומות שונים: העיר וההר. אם הכוונה לעיר, הויקידאטה הוא Q651583 והשם: הויקידאטה והקואורדינטות הנוכחיות ב-nli הן לא של etters-berg אלא של ettersburg הישוב. אם הכוונה היא להר, ממליצה לשנות את השם לאטרס-ברג (גרמניה: הר) והויקידאטה הוא  Q31547753</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>אלה הם שני מקומות שונים: העיר וההר. אם הכוונה לעיר, הויקידאטה הוא Q651583 והשם: הויקידאטה והקואורדינטות הנוכחיות ב-nli הן לא של etters-berg אלא של ettersburg הישוב. אם הכוונה היא להר, ממליצה לשנות את השם לאטרס-ברג (גרמניה: הר) והויקידאטה הוא  Q31547753</t>
+          <t>https://www.nli.org.il/he/authorities/987007561549805171</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007561549805171</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -10032,13 +10019,12 @@
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987007546333605171</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007546333605171</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -10086,13 +10072,12 @@
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987007284646705171</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007284646705171</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -10144,13 +10129,12 @@
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987007564769205171</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987007564769205171</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -10202,13 +10186,12 @@
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987011433524905171</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
-        <is>
-          <t>https://www.nli.org.il/he/authorities/987011433524905171</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -10256,20 +10239,19 @@
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.nli.org.il/he/authorities/987007545173905171</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://www.nli.org.il/he/authorities/987007545173905171</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
           <t>2026-09-22</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N9"/>
+  <autoFilter ref="A1:M9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>